<commit_message>
Wire home page import to the home-ecosystem block
Regenerate the home page via the import pipeline so content/index uses
the new home-ecosystem block instead of the old hero-partner +
cards-stats + cards-product combo. Add parsers/home-ecosystem.js
(title, description, check list, partner badge, metric rows) and point
import-home.js at a single .home-pn instance; rebundle.

Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/tools/importer/reports/import-home.report.xlsx
+++ b/tools/importer/reports/import-home.report.xlsx
@@ -79,7 +79,7 @@
     <t>index.report.json</t>
   </si>
   <si>
-    <t>["hero-partner","cards-stats","cards-product"]</t>
+    <t>["home-ecosystem"]</t>
   </si>
   <si>
     <t>index</t>
@@ -88,7 +88,7 @@
     <t>home</t>
   </si>
   <si>
-    <t>2026-08-26T00:00:32.615Z</t>
+    <t>2026-09-09T23:34:14.691Z</t>
   </si>
   <si>
     <t>http://adobe.puntos.net.s3-website-us-east-1.amazonaws.com/</t>

</xml_diff>